<commit_message>
Republish LaSeu_2025_WC: Kayak Cross individual (Time Trials) RANK from official classification (122 cells; maintainer 2026-10-21)
</commit_message>
<xml_diff>
--- a/events/LaSeu_2025_WC/LaSeu_2025_WC_start.xlsx
+++ b/events/LaSeu_2025_WC/LaSeu_2025_WC_start.xlsx
@@ -20335,6 +20335,11 @@
       <c r="K337" t="n">
         <v>336</v>
       </c>
+      <c r="M337" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R337" t="inlineStr">
         <is>
           <t>LOGACHEVA Taisiia</t>
@@ -20393,6 +20398,11 @@
       <c r="K338" t="n">
         <v>337</v>
       </c>
+      <c r="M338" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R338" t="inlineStr">
         <is>
           <t>MILLS Waris</t>
@@ -20456,6 +20466,11 @@
       <c r="K339" t="n">
         <v>338</v>
       </c>
+      <c r="M339" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R339" t="inlineStr">
         <is>
           <t>LUKNAROVA Emanuela</t>
@@ -20519,6 +20534,11 @@
       <c r="K340" t="n">
         <v>339</v>
       </c>
+      <c r="M340" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R340" t="inlineStr">
         <is>
           <t>KRYLOVA Kseniia</t>
@@ -20582,6 +20602,11 @@
       <c r="K341" t="n">
         <v>340</v>
       </c>
+      <c r="M341" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R341" t="inlineStr">
         <is>
           <t>MINAZOVA Alsu</t>
@@ -20708,6 +20733,11 @@
       <c r="K343" t="n">
         <v>342</v>
       </c>
+      <c r="M343" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R343" t="inlineStr">
         <is>
           <t>CHEN Lin</t>
@@ -20771,6 +20801,11 @@
       <c r="K344" t="n">
         <v>343</v>
       </c>
+      <c r="M344" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R344" t="inlineStr">
         <is>
           <t>HERZOG Andrea</t>
@@ -20834,6 +20869,11 @@
       <c r="K345" t="n">
         <v>344</v>
       </c>
+      <c r="M345" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R345" t="inlineStr">
         <is>
           <t>BAYN Nele</t>
@@ -20897,6 +20937,11 @@
       <c r="K346" t="n">
         <v>345</v>
       </c>
+      <c r="M346" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R346" t="inlineStr">
         <is>
           <t>OLSON Beatrice</t>
@@ -20960,6 +21005,11 @@
       <c r="K347" t="n">
         <v>346</v>
       </c>
+      <c r="M347" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R347" t="inlineStr">
         <is>
           <t>PITCHER FARRELL Cleo</t>
@@ -21023,6 +21073,11 @@
       <c r="K348" t="n">
         <v>347</v>
       </c>
+      <c r="M348" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R348" t="inlineStr">
         <is>
           <t>ARMANI Emilie</t>
@@ -21086,6 +21141,11 @@
       <c r="K349" t="n">
         <v>348</v>
       </c>
+      <c r="M349" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R349" t="inlineStr">
         <is>
           <t>SOMMERNES Iris</t>
@@ -21149,6 +21209,11 @@
       <c r="K350" t="n">
         <v>349</v>
       </c>
+      <c r="M350" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R350" t="inlineStr">
         <is>
           <t>MATTI Svenja</t>
@@ -21212,6 +21277,11 @@
       <c r="K351" t="n">
         <v>350</v>
       </c>
+      <c r="M351" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R351" t="inlineStr">
         <is>
           <t>PELLICER CHICA Laura</t>
@@ -21275,6 +21345,11 @@
       <c r="K352" t="n">
         <v>351</v>
       </c>
+      <c r="M352" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R352" t="inlineStr">
         <is>
           <t>WAN Shunfang</t>
@@ -21338,6 +21413,11 @@
       <c r="K353" t="n">
         <v>352</v>
       </c>
+      <c r="M353" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R353" t="inlineStr">
         <is>
           <t>SAMKOVA Olga</t>
@@ -21401,6 +21481,11 @@
       <c r="K354" t="n">
         <v>353</v>
       </c>
+      <c r="M354" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R354" t="inlineStr">
         <is>
           <t>GORA Aleksandra</t>
@@ -21464,6 +21549,11 @@
       <c r="K355" t="n">
         <v>354</v>
       </c>
+      <c r="M355" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R355" t="inlineStr">
         <is>
           <t>SORRIBES Laia</t>
@@ -21590,6 +21680,11 @@
       <c r="K357" t="n">
         <v>356</v>
       </c>
+      <c r="M357" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
       <c r="R357" t="inlineStr">
         <is>
           <t>LEAVER Lois</t>
@@ -21653,6 +21748,11 @@
       <c r="K358" t="n">
         <v>357</v>
       </c>
+      <c r="M358" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R358" t="inlineStr">
         <is>
           <t>BALDONI Lea</t>
@@ -21716,6 +21816,11 @@
       <c r="K359" t="n">
         <v>358</v>
       </c>
+      <c r="M359" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R359" t="inlineStr">
         <is>
           <t>O'CALLAGHAN Georgia</t>
@@ -21779,6 +21884,11 @@
       <c r="K360" t="n">
         <v>359</v>
       </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R360" t="inlineStr">
         <is>
           <t>ALTMAN Marcella</t>
@@ -21842,6 +21952,11 @@
       <c r="K361" t="n">
         <v>360</v>
       </c>
+      <c r="M361" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R361" t="inlineStr">
         <is>
           <t>PANKOVA Zuzana</t>
@@ -21905,6 +22020,11 @@
       <c r="K362" t="n">
         <v>361</v>
       </c>
+      <c r="M362" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R362" t="inlineStr">
         <is>
           <t>STANOVSKA Sona</t>
@@ -21968,6 +22088,11 @@
       <c r="K363" t="n">
         <v>362</v>
       </c>
+      <c r="M363" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R363" t="inlineStr">
         <is>
           <t>HILGERTOVA Amalie</t>
@@ -22031,6 +22156,11 @@
       <c r="K364" t="n">
         <v>363</v>
       </c>
+      <c r="M364" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R364" t="inlineStr">
         <is>
           <t>NOVAK Ajda</t>
@@ -22094,6 +22224,11 @@
       <c r="K365" t="n">
         <v>364</v>
       </c>
+      <c r="M365" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R365" t="inlineStr">
         <is>
           <t>SABATTINI Chiara</t>
@@ -22157,6 +22292,11 @@
       <c r="K366" t="n">
         <v>365</v>
       </c>
+      <c r="M366" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R366" t="inlineStr">
         <is>
           <t>HOCEVAR Eva Alina</t>
@@ -22220,6 +22360,11 @@
       <c r="K367" t="n">
         <v>366</v>
       </c>
+      <c r="M367" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R367" t="inlineStr">
         <is>
           <t>LAZKANO Miren</t>
@@ -22346,6 +22491,11 @@
       <c r="K369" t="n">
         <v>368</v>
       </c>
+      <c r="M369" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R369" t="inlineStr">
         <is>
           <t>XIE Xueting</t>
@@ -22409,6 +22559,11 @@
       <c r="K370" t="n">
         <v>369</v>
       </c>
+      <c r="M370" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R370" t="inlineStr">
         <is>
           <t>US Viktoriia</t>
@@ -22472,6 +22627,11 @@
       <c r="K371" t="n">
         <v>370</v>
       </c>
+      <c r="M371" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R371" t="inlineStr">
         <is>
           <t>KNEBLOVA Tereza</t>
@@ -22535,6 +22695,11 @@
       <c r="K372" t="n">
         <v>371</v>
       </c>
+      <c r="M372" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R372" t="inlineStr">
         <is>
           <t>DORIA Monica</t>
@@ -22598,6 +22763,11 @@
       <c r="K373" t="n">
         <v>372</v>
       </c>
+      <c r="M373" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R373" t="inlineStr">
         <is>
           <t>FOX Jessica</t>
@@ -22661,6 +22831,11 @@
       <c r="K374" t="n">
         <v>373</v>
       </c>
+      <c r="M374" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R374" t="inlineStr">
         <is>
           <t>SETCHELL Nikita</t>
@@ -22724,6 +22899,11 @@
       <c r="K375" t="n">
         <v>374</v>
       </c>
+      <c r="M375" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R375" t="inlineStr">
         <is>
           <t>VUITTON Emma</t>
@@ -22787,6 +22967,11 @@
       <c r="K376" t="n">
         <v>375</v>
       </c>
+      <c r="M376" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R376" t="inlineStr">
         <is>
           <t>LEIBFARTH Evy</t>
@@ -22850,6 +23035,11 @@
       <c r="K377" t="n">
         <v>376</v>
       </c>
+      <c r="M377" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R377" t="inlineStr">
         <is>
           <t>FUNK Ricarda</t>
@@ -22913,6 +23103,11 @@
       <c r="K378" t="n">
         <v>377</v>
       </c>
+      <c r="M378" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R378" t="inlineStr">
         <is>
           <t>MARX Alena</t>
@@ -22976,6 +23171,11 @@
       <c r="K379" t="n">
         <v>378</v>
       </c>
+      <c r="M379" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R379" t="inlineStr">
         <is>
           <t>CHOURRAUT Maialen</t>
@@ -23039,6 +23239,11 @@
       <c r="K380" t="n">
         <v>379</v>
       </c>
+      <c r="M380" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R380" t="inlineStr">
         <is>
           <t>FOX Noemie</t>
@@ -23102,6 +23307,11 @@
       <c r="K381" t="n">
         <v>380</v>
       </c>
+      <c r="M381" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R381" t="inlineStr">
         <is>
           <t>PRIGENT Camille</t>
@@ -23165,6 +23375,11 @@
       <c r="K382" t="n">
         <v>381</v>
       </c>
+      <c r="M382" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R382" t="inlineStr">
         <is>
           <t>HUG Angele</t>
@@ -23228,6 +23443,11 @@
       <c r="K383" t="n">
         <v>382</v>
       </c>
+      <c r="M383" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R383" t="inlineStr">
         <is>
           <t>WOODS Kimberley</t>
@@ -23291,6 +23511,11 @@
       <c r="K384" t="n">
         <v>383</v>
       </c>
+      <c r="M384" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
       <c r="R384" t="inlineStr">
         <is>
           <t>ISLAMOV Daniyar</t>
@@ -23354,6 +23579,11 @@
       <c r="K385" t="n">
         <v>384</v>
       </c>
+      <c r="M385" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
       <c r="R385" t="inlineStr">
         <is>
           <t>SMIRNOV Egor</t>
@@ -23480,6 +23710,11 @@
       <c r="K387" t="n">
         <v>386</v>
       </c>
+      <c r="M387" t="inlineStr">
+        <is>
+          <t>37</t>
+        </is>
+      </c>
       <c r="R387" t="inlineStr">
         <is>
           <t>EIGEL Pavel</t>
@@ -23543,6 +23778,11 @@
       <c r="K388" t="n">
         <v>387</v>
       </c>
+      <c r="M388" t="inlineStr">
+        <is>
+          <t>78</t>
+        </is>
+      </c>
       <c r="R388" t="inlineStr">
         <is>
           <t>ONG Jun Yi</t>
@@ -23606,6 +23846,11 @@
       <c r="K389" t="n">
         <v>388</v>
       </c>
+      <c r="M389" t="inlineStr">
+        <is>
+          <t>69</t>
+        </is>
+      </c>
       <c r="R389" t="inlineStr">
         <is>
           <t>NDIAYE Youssouf Wally</t>
@@ -23732,6 +23977,11 @@
       <c r="K391" t="n">
         <v>390</v>
       </c>
+      <c r="M391" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
       <c r="R391" t="inlineStr">
         <is>
           <t>GUBENKO Nikita</t>
@@ -23795,6 +24045,11 @@
       <c r="K392" t="n">
         <v>391</v>
       </c>
+      <c r="M392" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
       <c r="R392" t="inlineStr">
         <is>
           <t>KOZLOV Ivan</t>
@@ -23921,6 +24176,11 @@
       <c r="K394" t="n">
         <v>393</v>
       </c>
+      <c r="M394" t="inlineStr">
+        <is>
+          <t>42</t>
+        </is>
+      </c>
       <c r="R394" t="inlineStr">
         <is>
           <t>CHECA BARO Nil</t>
@@ -23984,6 +24244,11 @@
       <c r="K395" t="n">
         <v>394</v>
       </c>
+      <c r="M395" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
       <c r="R395" t="inlineStr">
         <is>
           <t>FRANCIS Nathaniel</t>
@@ -24047,6 +24312,11 @@
       <c r="K396" t="n">
         <v>395</v>
       </c>
+      <c r="M396" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
       <c r="R396" t="inlineStr">
         <is>
           <t>SNOOK George</t>
@@ -24110,6 +24380,11 @@
       <c r="K397" t="n">
         <v>396</v>
       </c>
+      <c r="M397" t="inlineStr">
+        <is>
+          <t>41</t>
+        </is>
+      </c>
       <c r="R397" t="inlineStr">
         <is>
           <t>MUTO Yusuke</t>
@@ -24173,6 +24448,11 @@
       <c r="K398" t="n">
         <v>397</v>
       </c>
+      <c r="M398" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
       <c r="R398" t="inlineStr">
         <is>
           <t>WEWEGE Donovan</t>
@@ -24236,6 +24516,11 @@
       <c r="K399" t="n">
         <v>398</v>
       </c>
+      <c r="M399" t="inlineStr">
+        <is>
+          <t>49</t>
+        </is>
+      </c>
       <c r="R399" t="inlineStr">
         <is>
           <t>TEMIRGALIEV Djanibek</t>
@@ -24299,6 +24584,11 @@
       <c r="K400" t="n">
         <v>399</v>
       </c>
+      <c r="M400" t="inlineStr">
+        <is>
+          <t>48</t>
+        </is>
+      </c>
       <c r="R400" t="inlineStr">
         <is>
           <t>STEINBRENNER Max</t>
@@ -24362,6 +24652,11 @@
       <c r="K401" t="n">
         <v>400</v>
       </c>
+      <c r="M401" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
       <c r="R401" t="inlineStr">
         <is>
           <t>MING Xingzhou</t>
@@ -24425,6 +24720,11 @@
       <c r="K402" t="n">
         <v>401</v>
       </c>
+      <c r="M402" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
       <c r="R402" t="inlineStr">
         <is>
           <t>LOCNIKAR Jan</t>
@@ -24488,6 +24788,11 @@
       <c r="K403" t="n">
         <v>402</v>
       </c>
+      <c r="M403" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
       <c r="R403" t="inlineStr">
         <is>
           <t>MAPELLI Guilherme</t>
@@ -24551,6 +24856,11 @@
       <c r="K404" t="n">
         <v>403</v>
       </c>
+      <c r="M404" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
       <c r="R404" t="inlineStr">
         <is>
           <t>ZHANG Hejie</t>
@@ -24614,6 +24924,11 @@
       <c r="K405" t="n">
         <v>404</v>
       </c>
+      <c r="M405" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
       <c r="R405" t="inlineStr">
         <is>
           <t>RUDORFER Martin</t>
@@ -24677,6 +24992,11 @@
       <c r="K406" t="n">
         <v>405</v>
       </c>
+      <c r="M406" t="inlineStr">
+        <is>
+          <t>77</t>
+        </is>
+      </c>
       <c r="R406" t="inlineStr">
         <is>
           <t>GONSENICA Adam</t>
@@ -24740,6 +25060,11 @@
       <c r="K407" t="n">
         <v>406</v>
       </c>
+      <c r="M407" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
       <c r="R407" t="inlineStr">
         <is>
           <t>TANAKA Yuuki</t>
@@ -24803,6 +25128,11 @@
       <c r="K408" t="n">
         <v>407</v>
       </c>
+      <c r="M408" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
       <c r="R408" t="inlineStr">
         <is>
           <t>CANO MOLE Luca</t>
@@ -24866,6 +25196,11 @@
       <c r="K409" t="n">
         <v>408</v>
       </c>
+      <c r="M409" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
       <c r="R409" t="inlineStr">
         <is>
           <t>EICHFELD Casey</t>
@@ -24929,6 +25264,11 @@
       <c r="K410" t="n">
         <v>409</v>
       </c>
+      <c r="M410" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
       <c r="R410" t="inlineStr">
         <is>
           <t>GRIGAR Jakub</t>
@@ -24992,6 +25332,11 @@
       <c r="K411" t="n">
         <v>410</v>
       </c>
+      <c r="M411" t="inlineStr">
+        <is>
+          <t>76</t>
+        </is>
+      </c>
       <c r="R411" t="inlineStr">
         <is>
           <t>ROZENTALS Klass Francisks</t>
@@ -25055,6 +25400,11 @@
       <c r="K412" t="n">
         <v>411</v>
       </c>
+      <c r="M412" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
       <c r="R412" t="inlineStr">
         <is>
           <t>HAYLETT Ben</t>
@@ -25118,6 +25468,11 @@
       <c r="K413" t="n">
         <v>412</v>
       </c>
+      <c r="M413" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
       <c r="R413" t="inlineStr">
         <is>
           <t>BARAT Andy</t>
@@ -25181,6 +25536,11 @@
       <c r="K414" t="n">
         <v>413</v>
       </c>
+      <c r="M414" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
       <c r="R414" t="inlineStr">
         <is>
           <t>SARAMANDIF Terence</t>
@@ -25244,6 +25604,11 @@
       <c r="K415" t="n">
         <v>414</v>
       </c>
+      <c r="M415" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
       <c r="R415" t="inlineStr">
         <is>
           <t>JACOB Lucas</t>
@@ -25307,6 +25672,11 @@
       <c r="K416" t="n">
         <v>415</v>
       </c>
+      <c r="M416" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
       <c r="R416" t="inlineStr">
         <is>
           <t>UKALOVIC Thomas</t>
@@ -25370,6 +25740,11 @@
       <c r="K417" t="n">
         <v>416</v>
       </c>
+      <c r="M417" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
       <c r="R417" t="inlineStr">
         <is>
           <t>HUANG Liman</t>
@@ -25433,6 +25808,11 @@
       <c r="K418" t="n">
         <v>417</v>
       </c>
+      <c r="M418" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
       <c r="R418" t="inlineStr">
         <is>
           <t>CUNHA Joao</t>
@@ -25496,6 +25876,11 @@
       <c r="K419" t="n">
         <v>418</v>
       </c>
+      <c r="M419" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
       <c r="R419" t="inlineStr">
         <is>
           <t>ZIELONKA Mark</t>
@@ -25559,6 +25944,11 @@
       <c r="K420" t="n">
         <v>419</v>
       </c>
+      <c r="M420" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
       <c r="R420" t="inlineStr">
         <is>
           <t>SOVKO Serhii</t>
@@ -25622,6 +26012,11 @@
       <c r="K421" t="n">
         <v>420</v>
       </c>
+      <c r="M421" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
       <c r="R421" t="inlineStr">
         <is>
           <t>BOYD Trevor</t>
@@ -25685,6 +26080,11 @@
       <c r="K422" t="n">
         <v>421</v>
       </c>
+      <c r="M422" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
       <c r="R422" t="inlineStr">
         <is>
           <t>JEGOU Liam</t>
@@ -25748,6 +26148,11 @@
       <c r="K423" t="n">
         <v>422</v>
       </c>
+      <c r="M423" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
       <c r="R423" t="inlineStr">
         <is>
           <t>PUCHNER Oliver</t>
@@ -25811,6 +26216,11 @@
       <c r="K424" t="n">
         <v>423</v>
       </c>
+      <c r="M424" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
       <c r="R424" t="inlineStr">
         <is>
           <t>TRIPANO Manuel</t>
@@ -25874,6 +26284,11 @@
       <c r="K425" t="n">
         <v>424</v>
       </c>
+      <c r="M425" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
       <c r="R425" t="inlineStr">
         <is>
           <t>FRIEDENSON Kaelin</t>
@@ -25937,6 +26352,11 @@
       <c r="K426" t="n">
         <v>425</v>
       </c>
+      <c r="M426" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
       <c r="R426" t="inlineStr">
         <is>
           <t>BRZEZINSKI Jakub</t>
@@ -26000,6 +26420,11 @@
       <c r="K427" t="n">
         <v>426</v>
       </c>
+      <c r="M427" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
       <c r="R427" t="inlineStr">
         <is>
           <t>ECHANIZ Pau</t>
@@ -26063,6 +26488,11 @@
       <c r="K428" t="n">
         <v>427</v>
       </c>
+      <c r="M428" t="inlineStr">
+        <is>
+          <t>51</t>
+        </is>
+      </c>
       <c r="R428" t="inlineStr">
         <is>
           <t>AUBERTIN Maxime</t>
@@ -26126,6 +26556,11 @@
       <c r="K429" t="n">
         <v>428</v>
       </c>
+      <c r="M429" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
       <c r="R429" t="inlineStr">
         <is>
           <t>NOVAK Matyas</t>
@@ -26189,6 +26624,11 @@
       <c r="K430" t="n">
         <v>429</v>
       </c>
+      <c r="M430" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
       <c r="R430" t="inlineStr">
         <is>
           <t>PASIUT Michal</t>
@@ -26252,6 +26692,11 @@
       <c r="K431" t="n">
         <v>430</v>
       </c>
+      <c r="M431" t="inlineStr">
+        <is>
+          <t>61</t>
+        </is>
+      </c>
       <c r="R431" t="inlineStr">
         <is>
           <t>MARTINEZ Jesus</t>
@@ -26315,6 +26760,11 @@
       <c r="K432" t="n">
         <v>431</v>
       </c>
+      <c r="M432" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
       <c r="R432" t="inlineStr">
         <is>
           <t>IVCHENKO Artem</t>
@@ -26378,6 +26828,11 @@
       <c r="K433" t="n">
         <v>432</v>
       </c>
+      <c r="M433" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
       <c r="R433" t="inlineStr">
         <is>
           <t>PEREZ RINCON Alexis</t>
@@ -26441,6 +26896,11 @@
       <c r="K434" t="n">
         <v>433</v>
       </c>
+      <c r="M434" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
       <c r="R434" t="inlineStr">
         <is>
           <t>SAVLI Jakob</t>
@@ -26504,6 +26964,11 @@
       <c r="K435" t="n">
         <v>434</v>
       </c>
+      <c r="M435" t="inlineStr">
+        <is>
+          <t>35</t>
+        </is>
+      </c>
       <c r="R435" t="inlineStr">
         <is>
           <t>ALVARENGA Frederico</t>
@@ -26567,6 +27032,11 @@
       <c r="K436" t="n">
         <v>435</v>
       </c>
+      <c r="M436" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
       <c r="R436" t="inlineStr">
         <is>
           <t>MCCREERY Alistair</t>
@@ -26630,6 +27100,11 @@
       <c r="K437" t="n">
         <v>436</v>
       </c>
+      <c r="M437" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
       <c r="R437" t="inlineStr">
         <is>
           <t>HALCIN Martin</t>
@@ -26693,6 +27168,11 @@
       <c r="K438" t="n">
         <v>437</v>
       </c>
+      <c r="M438" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
       <c r="R438" t="inlineStr">
         <is>
           <t>POPE Benjamin</t>
@@ -26756,6 +27236,11 @@
       <c r="K439" t="n">
         <v>438</v>
       </c>
+      <c r="M439" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
       <c r="R439" t="inlineStr">
         <is>
           <t>ROELLER Tillmann</t>
@@ -26819,6 +27304,11 @@
       <c r="K440" t="n">
         <v>439</v>
       </c>
+      <c r="M440" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
       <c r="R440" t="inlineStr">
         <is>
           <t>OHRSTROM Isak</t>
@@ -26945,6 +27435,11 @@
       <c r="K442" t="n">
         <v>441</v>
       </c>
+      <c r="M442" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
       <c r="R442" t="inlineStr">
         <is>
           <t>DESNOS Mathieu</t>
@@ -27008,6 +27503,11 @@
       <c r="K443" t="n">
         <v>442</v>
       </c>
+      <c r="M443" t="inlineStr">
+        <is>
+          <t>74</t>
+        </is>
+      </c>
       <c r="R443" t="inlineStr">
         <is>
           <t>BALDONI Alex</t>
@@ -27071,6 +27571,11 @@
       <c r="K444" t="n">
         <v>443</v>
       </c>
+      <c r="M444" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
       <c r="R444" t="inlineStr">
         <is>
           <t>DE COSTER Gabriel</t>
@@ -27134,6 +27639,11 @@
       <c r="K445" t="n">
         <v>444</v>
       </c>
+      <c r="M445" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
       <c r="R445" t="inlineStr">
         <is>
           <t>HENGST Stefan</t>
@@ -27197,6 +27707,11 @@
       <c r="K446" t="n">
         <v>445</v>
       </c>
+      <c r="M446" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="R446" t="inlineStr">
         <is>
           <t>KREJCI Jakub</t>
@@ -27260,6 +27775,11 @@
       <c r="K447" t="n">
         <v>446</v>
       </c>
+      <c r="M447" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
       <c r="R447" t="inlineStr">
         <is>
           <t>HOCEVAR Ziga Lin</t>
@@ -27323,6 +27843,11 @@
       <c r="K448" t="n">
         <v>447</v>
       </c>
+      <c r="M448" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
       <c r="R448" t="inlineStr">
         <is>
           <t>DELFOUR Lucien</t>
@@ -27386,6 +27911,11 @@
       <c r="K449" t="n">
         <v>448</v>
       </c>
+      <c r="M449" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
       <c r="R449" t="inlineStr">
         <is>
           <t>OSCHMAUTZ Felix</t>
@@ -27449,6 +27979,11 @@
       <c r="K450" t="n">
         <v>449</v>
       </c>
+      <c r="M450" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
       <c r="R450" t="inlineStr">
         <is>
           <t>CASTRYCK Titouan</t>
@@ -27512,6 +28047,11 @@
       <c r="K451" t="n">
         <v>450</v>
       </c>
+      <c r="M451" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
       <c r="R451" t="inlineStr">
         <is>
           <t>LEAVER Sam</t>
@@ -27575,6 +28115,11 @@
       <c r="K452" t="n">
         <v>451</v>
       </c>
+      <c r="M452" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
       <c r="R452" t="inlineStr">
         <is>
           <t>ANDERSON Timothy</t>
@@ -27638,6 +28183,11 @@
       <c r="K453" t="n">
         <v>452</v>
       </c>
+      <c r="M453" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="R453" t="inlineStr">
         <is>
           <t>DICKSON Jonny</t>
@@ -27701,6 +28251,11 @@
       <c r="K454" t="n">
         <v>453</v>
       </c>
+      <c r="M454" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
       <c r="R454" t="inlineStr">
         <is>
           <t>ECHEVERRIA OLGUIN Andraz</t>
@@ -27764,6 +28319,11 @@
       <c r="K455" t="n">
         <v>454</v>
       </c>
+      <c r="M455" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="R455" t="inlineStr">
         <is>
           <t>ROHRER Jan</t>
@@ -27827,6 +28387,11 @@
       <c r="K456" t="n">
         <v>455</v>
       </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="R456" t="inlineStr">
         <is>
           <t>MADORE Mathurin</t>
@@ -27890,6 +28455,11 @@
       <c r="K457" t="n">
         <v>456</v>
       </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
       <c r="R457" t="inlineStr">
         <is>
           <t>GONCALVES Pedro</t>
@@ -27953,6 +28523,11 @@
       <c r="K458" t="n">
         <v>457</v>
       </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="R458" t="inlineStr">
         <is>
           <t>OCHOA Manuel</t>
@@ -28016,6 +28591,11 @@
       <c r="K459" t="n">
         <v>458</v>
       </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
       <c r="R459" t="inlineStr">
         <is>
           <t>HEGGE Noah</t>
@@ -28079,6 +28659,11 @@
       <c r="K460" t="n">
         <v>459</v>
       </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
       <c r="R460" t="inlineStr">
         <is>
           <t>POLACZYK Mateusz</t>
@@ -28142,6 +28727,11 @@
       <c r="K461" t="n">
         <v>460</v>
       </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
       <c r="R461" t="inlineStr">
         <is>
           <t>LLORENTE David</t>
@@ -28205,6 +28795,11 @@
       <c r="K462" t="n">
         <v>461</v>
       </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
       <c r="R462" t="inlineStr">
         <is>
           <t>RENIA Benjamin</t>
@@ -28268,6 +28863,11 @@
       <c r="K463" t="n">
         <v>462</v>
       </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
       <c r="R463" t="inlineStr">
         <is>
           <t>MARX Dimitri</t>
@@ -28331,6 +28931,11 @@
       <c r="K464" t="n">
         <v>463</v>
       </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>46</t>
+        </is>
+      </c>
       <c r="R464" t="inlineStr">
         <is>
           <t>DOUGOUD Martin</t>
@@ -28393,6 +28998,11 @@
       </c>
       <c r="K465" t="n">
         <v>464</v>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="R465" t="inlineStr">
         <is>

</xml_diff>